<commit_message>
docs(pid): grafa o docente como Douglas de Oliveira Matos Braga
A planilha institucional de rotinas traz "DOUGLAS DE OLIVEIRA MATOS", mas
o nome em uso no livro e no e-mail institucional inclui o sobrenome Braga.
Ajusta o campo de docente responsável e a entrada de referência do próprio
material didático (ABNT: BRAGA, Douglas de Oliveira Matos).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014SkoDLvPhyuziAgagUgqdq
</commit_message>
<xml_diff>
--- a/atividades/PID - Bases de Ciencia da Computacao 5 - 2.2026.xlsx
+++ b/atividades/PID - Bases de Ciencia da Computacao 5 - 2.2026.xlsx
@@ -1019,7 +1019,7 @@
       </c>
       <c r="B8" s="49" t="inlineStr">
         <is>
-          <t>Douglas de Oliveira Matos</t>
+          <t>Douglas de Oliveira Matos Braga</t>
         </is>
       </c>
       <c r="C8" s="50" t="n"/>
@@ -1727,7 +1727,7 @@
           <t>BÁSICA
 GRUS, Joel. Data science do zero: noções fundamentais com Python. 2. ed. Rio de Janeiro: Alta Books, 2021.
 GRUS, Joel. Data science from scratch: first principles with Python. 2nd ed. Sebastopol: O'Reilly Media, 2019.
-MATOS, Douglas de Oliveira. Bases de Ciência da Computação 5: ciência de dados. Brasília: UnDF, 2026. Material didático da unidade curricular. Disponível em: https://bragad.github.io/UnDF-Bases5-CienciaDeDados-202602/
+BRAGA, Douglas de Oliveira Matos. Bases de Ciência da Computação 5: ciência de dados. Brasília: UnDF, 2026. Material didático da unidade curricular. Disponível em: https://bragad.github.io/UnDF-Bases5-CienciaDeDados-202602/
 COMPLEMENTAR
 GÉRON, Aurélien. Mãos à obra: aprendizado de máquina com Scikit-Learn, Keras &amp; TensorFlow. 2. ed. Rio de Janeiro: Alta Books, 2021.
 VANDERPLAS, Jake. Python data science handbook: essential tools for working with data. 2nd ed. Sebastopol: O'Reilly Media, 2023.

</xml_diff>